<commit_message>
refactor: MECE cleanup - remove 327-line dead Section 4 from etl_pipeline, update README and DEV_LOG
</commit_message>
<xml_diff>
--- a/public/DataExtract/2026品檢報表統計.xlsx
+++ b/public/DataExtract/2026品檢報表統計.xlsx
@@ -3473,42 +3473,12 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S15"/>
+  <dimension ref="A1:N15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
         <v>原物料進料品檢</v>
       </c>
-      <c r="B1" t="str">
-        <v/>
-      </c>
-      <c r="C1" t="str">
-        <v/>
-      </c>
-      <c r="D1" t="str">
-        <v/>
-      </c>
-      <c r="E1" t="str">
-        <v/>
-      </c>
-      <c r="F1" t="str">
-        <v/>
-      </c>
-      <c r="G1" t="str">
-        <v/>
-      </c>
-      <c r="H1" t="str">
-        <v/>
-      </c>
-      <c r="I1" t="str">
-        <v/>
-      </c>
-      <c r="J1" t="str">
-        <v/>
-      </c>
-      <c r="K1" t="str">
-        <v>物料</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -3518,54 +3488,39 @@
         <v>原料</v>
       </c>
       <c r="C2" t="str">
-        <v>物料</v>
+        <v>B膠</v>
       </c>
       <c r="D2" t="str">
+        <v>收縮膜</v>
+      </c>
+      <c r="E2" t="str">
+        <v>色粉</v>
+      </c>
+      <c r="F2" t="str">
+        <v>空白包裝袋</v>
+      </c>
+      <c r="G2" t="str">
+        <v>空白感壓紙</v>
+      </c>
+      <c r="H2" t="str">
+        <v>塑膠袋</v>
+      </c>
+      <c r="I2" t="str">
+        <v>塑膠袋40*50</v>
+      </c>
+      <c r="J2" t="str">
         <v>紙箱</v>
       </c>
-      <c r="E2" t="str">
+      <c r="K2" t="str">
         <v>過濾網連蓋</v>
       </c>
-      <c r="F2" t="str">
+      <c r="L2" t="str">
         <v>標籤</v>
       </c>
-      <c r="G2" t="str">
+      <c r="M2" t="str">
         <v>射出D</v>
       </c>
-      <c r="H2" t="str">
-        <v>小計</v>
-      </c>
-      <c r="I2" t="str">
-        <v/>
-      </c>
-      <c r="J2" t="str">
-        <v/>
-      </c>
-      <c r="K2" t="str">
-        <v>月份</v>
-      </c>
-      <c r="L2" t="str">
-        <v>B膠</v>
-      </c>
-      <c r="M2" t="str">
-        <v>收縮膜</v>
-      </c>
       <c r="N2" t="str">
-        <v>色粉</v>
-      </c>
-      <c r="O2" t="str">
-        <v>空白包裝袋</v>
-      </c>
-      <c r="P2" t="str">
-        <v>空白感壓紙</v>
-      </c>
-      <c r="Q2" t="str">
-        <v>塑膠袋</v>
-      </c>
-      <c r="R2" t="str">
-        <v>塑膠袋40*50</v>
-      </c>
-      <c r="S2" t="str">
         <v>小計</v>
       </c>
     </row>
@@ -3577,55 +3532,40 @@
         <v>18</v>
       </c>
       <c r="C3">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="D3">
         <v>3</v>
       </c>
       <c r="E3">
+        <v>0</v>
+      </c>
+      <c r="F3">
+        <v>0</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <v>3</v>
+      </c>
+      <c r="I3">
+        <v>2</v>
+      </c>
+      <c r="J3">
+        <v>3</v>
+      </c>
+      <c r="K3">
         <v>15</v>
       </c>
-      <c r="F3">
-        <v>3</v>
-      </c>
-      <c r="G3">
+      <c r="L3">
+        <v>3</v>
+      </c>
+      <c r="M3">
         <v>181</v>
       </c>
-      <c r="H3">
+      <c r="N3">
         <v>228</v>
-      </c>
-      <c r="I3" t="str">
-        <v/>
-      </c>
-      <c r="J3" t="str">
-        <v/>
-      </c>
-      <c r="K3">
-        <v>1</v>
-      </c>
-      <c r="L3">
-        <v>0</v>
-      </c>
-      <c r="M3">
-        <v>3</v>
-      </c>
-      <c r="N3">
-        <v>0</v>
-      </c>
-      <c r="O3">
-        <v>0</v>
-      </c>
-      <c r="P3">
-        <v>0</v>
-      </c>
-      <c r="Q3">
-        <v>3</v>
-      </c>
-      <c r="R3">
-        <v>2</v>
-      </c>
-      <c r="S3">
-        <v>8</v>
       </c>
     </row>
     <row r="4">
@@ -3636,55 +3576,40 @@
         <v>6</v>
       </c>
       <c r="C4">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="D4">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E4">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4">
         <v>2</v>
       </c>
-      <c r="G4">
+      <c r="I4">
+        <v>1</v>
+      </c>
+      <c r="J4">
+        <v>3</v>
+      </c>
+      <c r="K4">
+        <v>0</v>
+      </c>
+      <c r="L4">
+        <v>2</v>
+      </c>
+      <c r="M4">
         <v>114</v>
       </c>
-      <c r="H4">
+      <c r="N4">
         <v>132</v>
-      </c>
-      <c r="I4" t="str">
-        <v/>
-      </c>
-      <c r="J4" t="str">
-        <v/>
-      </c>
-      <c r="K4">
-        <v>2</v>
-      </c>
-      <c r="L4">
-        <v>0</v>
-      </c>
-      <c r="M4">
-        <v>0</v>
-      </c>
-      <c r="N4">
-        <v>4</v>
-      </c>
-      <c r="O4">
-        <v>0</v>
-      </c>
-      <c r="P4">
-        <v>0</v>
-      </c>
-      <c r="Q4">
-        <v>2</v>
-      </c>
-      <c r="R4">
-        <v>1</v>
-      </c>
-      <c r="S4">
-        <v>7</v>
       </c>
     </row>
     <row r="5">
@@ -3695,55 +3620,40 @@
         <v>31</v>
       </c>
       <c r="C5">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5">
+        <v>2</v>
+      </c>
+      <c r="F5">
+        <v>0</v>
+      </c>
+      <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="H5">
+        <v>2</v>
+      </c>
+      <c r="I5">
+        <v>2</v>
+      </c>
+      <c r="J5">
         <v>4</v>
       </c>
-      <c r="E5">
-        <v>0</v>
-      </c>
-      <c r="F5">
-        <v>0</v>
-      </c>
-      <c r="G5">
+      <c r="K5">
+        <v>0</v>
+      </c>
+      <c r="L5">
+        <v>0</v>
+      </c>
+      <c r="M5">
         <v>217</v>
       </c>
-      <c r="H5">
+      <c r="N5">
         <v>258</v>
-      </c>
-      <c r="I5" t="str">
-        <v/>
-      </c>
-      <c r="J5" t="str">
-        <v/>
-      </c>
-      <c r="K5">
-        <v>3</v>
-      </c>
-      <c r="L5">
-        <v>0</v>
-      </c>
-      <c r="M5">
-        <v>0</v>
-      </c>
-      <c r="N5">
-        <v>2</v>
-      </c>
-      <c r="O5">
-        <v>0</v>
-      </c>
-      <c r="P5">
-        <v>0</v>
-      </c>
-      <c r="Q5">
-        <v>2</v>
-      </c>
-      <c r="R5">
-        <v>2</v>
-      </c>
-      <c r="S5">
-        <v>6</v>
       </c>
     </row>
     <row r="6">
@@ -3754,55 +3664,40 @@
         <v>16</v>
       </c>
       <c r="C6">
+        <v>0</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6">
+        <v>1</v>
+      </c>
+      <c r="F6">
+        <v>0</v>
+      </c>
+      <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6">
+        <v>2</v>
+      </c>
+      <c r="I6">
+        <v>2</v>
+      </c>
+      <c r="J6">
         <v>5</v>
       </c>
-      <c r="D6">
-        <v>5</v>
-      </c>
-      <c r="E6">
-        <v>0</v>
-      </c>
-      <c r="F6">
+      <c r="K6">
+        <v>0</v>
+      </c>
+      <c r="L6">
         <v>8</v>
       </c>
-      <c r="G6">
+      <c r="M6">
         <v>192</v>
       </c>
-      <c r="H6">
+      <c r="N6">
         <v>226</v>
-      </c>
-      <c r="I6" t="str">
-        <v/>
-      </c>
-      <c r="J6" t="str">
-        <v/>
-      </c>
-      <c r="K6">
-        <v>4</v>
-      </c>
-      <c r="L6">
-        <v>0</v>
-      </c>
-      <c r="M6">
-        <v>0</v>
-      </c>
-      <c r="N6">
-        <v>1</v>
-      </c>
-      <c r="O6">
-        <v>0</v>
-      </c>
-      <c r="P6">
-        <v>0</v>
-      </c>
-      <c r="Q6">
-        <v>2</v>
-      </c>
-      <c r="R6">
-        <v>2</v>
-      </c>
-      <c r="S6">
-        <v>5</v>
       </c>
     </row>
     <row r="7">
@@ -3813,55 +3708,40 @@
         <v>21</v>
       </c>
       <c r="C7">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D7">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F7">
+        <v>0</v>
+      </c>
+      <c r="G7">
+        <v>0</v>
+      </c>
+      <c r="H7">
+        <v>0</v>
+      </c>
+      <c r="I7">
         <v>1</v>
       </c>
-      <c r="G7">
+      <c r="J7">
+        <v>3</v>
+      </c>
+      <c r="K7">
+        <v>0</v>
+      </c>
+      <c r="L7">
+        <v>1</v>
+      </c>
+      <c r="M7">
         <v>193</v>
       </c>
-      <c r="H7">
+      <c r="N7">
         <v>220</v>
-      </c>
-      <c r="I7" t="str">
-        <v/>
-      </c>
-      <c r="J7" t="str">
-        <v/>
-      </c>
-      <c r="K7">
-        <v>5</v>
-      </c>
-      <c r="L7">
-        <v>0</v>
-      </c>
-      <c r="M7">
-        <v>0</v>
-      </c>
-      <c r="N7">
-        <v>1</v>
-      </c>
-      <c r="O7">
-        <v>0</v>
-      </c>
-      <c r="P7">
-        <v>0</v>
-      </c>
-      <c r="Q7">
-        <v>0</v>
-      </c>
-      <c r="R7">
-        <v>1</v>
-      </c>
-      <c r="S7">
-        <v>2</v>
       </c>
     </row>
     <row r="8">
@@ -3872,55 +3752,40 @@
         <v>9</v>
       </c>
       <c r="C8">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D8">
+        <v>0</v>
+      </c>
+      <c r="E8">
         <v>1</v>
       </c>
-      <c r="E8">
-        <v>0</v>
-      </c>
       <c r="F8">
+        <v>0</v>
+      </c>
+      <c r="G8">
+        <v>0</v>
+      </c>
+      <c r="H8">
         <v>1</v>
       </c>
-      <c r="G8">
+      <c r="I8">
+        <v>1</v>
+      </c>
+      <c r="J8">
+        <v>1</v>
+      </c>
+      <c r="K8">
+        <v>0</v>
+      </c>
+      <c r="L8">
+        <v>1</v>
+      </c>
+      <c r="M8">
         <v>86</v>
       </c>
-      <c r="H8">
+      <c r="N8">
         <v>100</v>
-      </c>
-      <c r="I8" t="str">
-        <v/>
-      </c>
-      <c r="J8" t="str">
-        <v/>
-      </c>
-      <c r="K8">
-        <v>6</v>
-      </c>
-      <c r="L8">
-        <v>0</v>
-      </c>
-      <c r="M8">
-        <v>0</v>
-      </c>
-      <c r="N8">
-        <v>1</v>
-      </c>
-      <c r="O8">
-        <v>0</v>
-      </c>
-      <c r="P8">
-        <v>0</v>
-      </c>
-      <c r="Q8">
-        <v>1</v>
-      </c>
-      <c r="R8">
-        <v>1</v>
-      </c>
-      <c r="S8">
-        <v>3</v>
       </c>
     </row>
     <row r="9">
@@ -3948,14 +3813,14 @@
       <c r="H9">
         <v>0</v>
       </c>
-      <c r="I9" t="str">
-        <v/>
-      </c>
-      <c r="J9" t="str">
-        <v/>
+      <c r="I9">
+        <v>0</v>
+      </c>
+      <c r="J9">
+        <v>0</v>
       </c>
       <c r="K9">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="L9">
         <v>0</v>
@@ -3964,21 +3829,6 @@
         <v>0</v>
       </c>
       <c r="N9">
-        <v>0</v>
-      </c>
-      <c r="O9">
-        <v>0</v>
-      </c>
-      <c r="P9">
-        <v>0</v>
-      </c>
-      <c r="Q9">
-        <v>0</v>
-      </c>
-      <c r="R9">
-        <v>0</v>
-      </c>
-      <c r="S9">
         <v>0</v>
       </c>
     </row>
@@ -4007,14 +3857,14 @@
       <c r="H10">
         <v>0</v>
       </c>
-      <c r="I10" t="str">
-        <v/>
-      </c>
-      <c r="J10" t="str">
-        <v/>
+      <c r="I10">
+        <v>0</v>
+      </c>
+      <c r="J10">
+        <v>0</v>
       </c>
       <c r="K10">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="L10">
         <v>0</v>
@@ -4023,21 +3873,6 @@
         <v>0</v>
       </c>
       <c r="N10">
-        <v>0</v>
-      </c>
-      <c r="O10">
-        <v>0</v>
-      </c>
-      <c r="P10">
-        <v>0</v>
-      </c>
-      <c r="Q10">
-        <v>0</v>
-      </c>
-      <c r="R10">
-        <v>0</v>
-      </c>
-      <c r="S10">
         <v>0</v>
       </c>
     </row>
@@ -4066,14 +3901,14 @@
       <c r="H11">
         <v>0</v>
       </c>
-      <c r="I11" t="str">
-        <v/>
-      </c>
-      <c r="J11" t="str">
-        <v/>
+      <c r="I11">
+        <v>0</v>
+      </c>
+      <c r="J11">
+        <v>0</v>
       </c>
       <c r="K11">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="L11">
         <v>0</v>
@@ -4082,21 +3917,6 @@
         <v>0</v>
       </c>
       <c r="N11">
-        <v>0</v>
-      </c>
-      <c r="O11">
-        <v>0</v>
-      </c>
-      <c r="P11">
-        <v>0</v>
-      </c>
-      <c r="Q11">
-        <v>0</v>
-      </c>
-      <c r="R11">
-        <v>0</v>
-      </c>
-      <c r="S11">
         <v>0</v>
       </c>
     </row>
@@ -4125,14 +3945,14 @@
       <c r="H12">
         <v>0</v>
       </c>
-      <c r="I12" t="str">
-        <v/>
-      </c>
-      <c r="J12" t="str">
-        <v/>
+      <c r="I12">
+        <v>0</v>
+      </c>
+      <c r="J12">
+        <v>0</v>
       </c>
       <c r="K12">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="L12">
         <v>0</v>
@@ -4141,21 +3961,6 @@
         <v>0</v>
       </c>
       <c r="N12">
-        <v>0</v>
-      </c>
-      <c r="O12">
-        <v>0</v>
-      </c>
-      <c r="P12">
-        <v>0</v>
-      </c>
-      <c r="Q12">
-        <v>0</v>
-      </c>
-      <c r="R12">
-        <v>0</v>
-      </c>
-      <c r="S12">
         <v>0</v>
       </c>
     </row>
@@ -4182,39 +3987,24 @@
         <v>0</v>
       </c>
       <c r="H13">
-        <v>4</v>
-      </c>
-      <c r="I13" t="str">
-        <v/>
-      </c>
-      <c r="J13" t="str">
-        <v/>
+        <v>0</v>
+      </c>
+      <c r="I13">
+        <v>0</v>
+      </c>
+      <c r="J13">
+        <v>0</v>
       </c>
       <c r="K13">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="L13">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="M13">
         <v>0</v>
       </c>
       <c r="N13">
-        <v>0</v>
-      </c>
-      <c r="O13">
-        <v>0</v>
-      </c>
-      <c r="P13">
-        <v>0</v>
-      </c>
-      <c r="Q13">
-        <v>0</v>
-      </c>
-      <c r="R13">
-        <v>0</v>
-      </c>
-      <c r="S13">
         <v>4</v>
       </c>
     </row>
@@ -4243,14 +4033,14 @@
       <c r="H14">
         <v>0</v>
       </c>
-      <c r="I14" t="str">
-        <v/>
-      </c>
-      <c r="J14" t="str">
-        <v/>
+      <c r="I14">
+        <v>0</v>
+      </c>
+      <c r="J14">
+        <v>0</v>
       </c>
       <c r="K14">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="L14">
         <v>0</v>
@@ -4259,21 +4049,6 @@
         <v>0</v>
       </c>
       <c r="N14">
-        <v>0</v>
-      </c>
-      <c r="O14">
-        <v>0</v>
-      </c>
-      <c r="P14">
-        <v>0</v>
-      </c>
-      <c r="Q14">
-        <v>0</v>
-      </c>
-      <c r="R14">
-        <v>0</v>
-      </c>
-      <c r="S14">
         <v>0</v>
       </c>
     </row>
@@ -4285,60 +4060,45 @@
         <v>101</v>
       </c>
       <c r="C15">
-        <v>35</v>
+        <v>4</v>
       </c>
       <c r="D15">
+        <v>3</v>
+      </c>
+      <c r="E15">
+        <v>9</v>
+      </c>
+      <c r="F15">
+        <v>0</v>
+      </c>
+      <c r="G15">
+        <v>0</v>
+      </c>
+      <c r="H15">
+        <v>10</v>
+      </c>
+      <c r="I15">
+        <v>9</v>
+      </c>
+      <c r="J15">
         <v>19</v>
       </c>
-      <c r="E15">
+      <c r="K15">
         <v>15</v>
       </c>
-      <c r="F15">
+      <c r="L15">
         <v>15</v>
       </c>
-      <c r="G15">
+      <c r="M15">
         <v>983</v>
       </c>
-      <c r="H15">
+      <c r="N15">
         <v>1168</v>
-      </c>
-      <c r="I15" t="str">
-        <v/>
-      </c>
-      <c r="J15" t="str">
-        <v/>
-      </c>
-      <c r="K15" t="str">
-        <v>小計</v>
-      </c>
-      <c r="L15">
-        <v>4</v>
-      </c>
-      <c r="M15">
-        <v>3</v>
-      </c>
-      <c r="N15">
-        <v>9</v>
-      </c>
-      <c r="O15">
-        <v>0</v>
-      </c>
-      <c r="P15">
-        <v>0</v>
-      </c>
-      <c r="Q15">
-        <v>10</v>
-      </c>
-      <c r="R15">
-        <v>9</v>
-      </c>
-      <c r="S15">
-        <v>35</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:S15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N15"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>